<commit_message>
feat: kolom alat untuk 22 pemeriksaan di kartu kerja sederhana
</commit_message>
<xml_diff>
--- a/testing/kertas-kerja/contoh-pengisian.xlsx
+++ b/testing/kertas-kerja/contoh-pengisian.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -550,101 +550,113 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Angka menunjukkan nomor pemeriksaan dari daftar 22 pemeriksaan. L berarti Lolos, G berarti Gagal, T berarti Tidak berlaku.</t>
+          <t>Kolom Alat yang dipakai menjelaskan alat untuk setiap baris. Kolom paling kiri adalah nomor pemeriksaan dari daftar 22 pemeriksaan. L berarti Lolos, G berarti Gagal, T berarti Tidak berlaku.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Contoh tanda G</t>
+          <t>Alat yang paling sering dipakai</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Tanda G selalu harus punya baris di sheet Daftar Temuan. Kolom Halaman diisi nomor halaman dari sheet Daftar Halaman.</t>
+          <t>Keyboard dan NVDA. DevTools hanya dipakai untuk melihat kode dan nama tombol. Perekam layar dipakai sebagai bukti.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Contoh tanda T</t>
+          <t>Contoh tanda G</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>T dipakai kalau fiturnya memang tidak ada di halaman itu. Contohnya halaman tanpa formulir tidak punya baris pesan kesalahan.</t>
+          <t>Tanda G selalu harus punya baris di sheet Daftar Temuan. Kolom Halaman diisi nomor halaman dari sheet Daftar Halaman.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nomor halaman</t>
+          <t>Contoh tanda T</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Buka sheet Daftar Halaman, kolom No. Halaman beranda bernomor 1.</t>
+          <t>T dipakai kalau fiturnya memang tidak ada di halaman itu. Contohnya halaman tanpa formulir tidak punya baris pesan kesalahan.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tingkat kerugian</t>
+          <t>Nomor halaman</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Serius berarti orang bisa menyelesaikan tugasnya tapi sangat susah. Bukan Sangat serius, karena halamannya masih bisa dipakai.</t>
+          <t>Buka sheet Daftar Halaman, kolom No. Halaman beranda bernomor 1.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Cara mengecek</t>
+          <t>Tingkat kerugian</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Tulis langkah yang bisa diulang orang lain tanpa perlu bertanya. Sebutkan kombinasi tombol dan apa yang didengar.</t>
+          <t>Serius berarti orang bisa menyelesaikan tugasnya tapi sangat susah. Bukan Sangat serius, karena halamannya masih bisa dipakai.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Nama berkas bukti</t>
+          <t>Cara mengecek</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Bukti disimpan di folder results/manual/evidence/ dengan nama yang sama seperti ditulis di kolom ini.</t>
+          <t>Tulis langkah yang bisa diulang orang lain tanpa perlu bertanya. Sebutkan kombinasi tombol dan apa yang didengar.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Kolom Sudah Diperiksa</t>
+          <t>Nama berkas bukti</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Diisi Koordinator. Ya berarti sudah diperiksa dan setuju, Belum berarti masih menunggu.</t>
+          <t>Bukti disimpan di folder results/manual/evidence/ dengan nama yang sama seperti ditulis di kolom ini.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>Kolom Sudah Diperiksa</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Diisi Koordinator. Ya berarti sudah diperiksa dan setuju, Belum berarti masih menunggu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>Contoh isi sheet Rekap</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Jumlah Gagal dan Jumlah Diuji dihitung otomatis dari tanda di sheet uji.</t>
         </is>
@@ -750,7 +762,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>beranda (Indonesia)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -760,7 +772,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>https://www.inovasi.or.id/en/</t>
+          <t>https://www.inovasi.or.id/</t>
         </is>
       </c>
       <c r="E4" s="5" t="n"/>
@@ -801,7 +813,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>nurturing-the-first-steps-of-readi</t>
+          <t>beranda (Inggris)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -811,7 +823,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>https://www.inovasi.or.id/en/publication/nurturing-the-first-steps-of-reading-in-cirebon</t>
+          <t>https://www.inovasi.or.id/en/</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -2489,14 +2501,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -2512,17 +2525,22 @@
           <t>Yang diperiksa</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Alat yang dipakai</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Halaman 1</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Halaman 2</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Halaman 10</t>
         </is>
@@ -2539,9 +2557,14 @@
           <t>Yang diperiksa</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n"/>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Alat yang dipakai</t>
+        </is>
+      </c>
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -2552,9 +2575,9 @@
           <t>Semua tombol bisa dipakai pakai keyboard saja</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Keyboard saja (Tab, Shift+Tab, Enter, Spasi, Esc, tombol panah). Tetikus tidak dipakai.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -2563,6 +2586,11 @@
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2577,9 +2605,9 @@
           <t>Tidak terjebak di dalam galeri, menu, atau searching</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Keyboard saja + perekam layar (Windows: Win+Alt+R)</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -2588,6 +2616,11 @@
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2602,9 +2635,9 @@
           <t>Urutan fokus masuk akal, mengikuti urutan yang dilihat mata</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Keyboard + DevTools: klik kanan elemen, pilih Inspect</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -2613,6 +2646,11 @@
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2627,9 +2665,9 @@
           <t>Kotak fokus terlihat jelas saat memakai keyboard</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Perekam layar + DevTools tab Accessibility</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -2638,6 +2676,11 @@
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2652,9 +2695,9 @@
           <t>Ada tombol lompat langsung ke konten utama</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Keyboard saja. Tekan Tab sekali di awal halaman.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -2663,6 +2706,11 @@
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2677,17 +2725,22 @@
           <t>Hanya ada satu bagian header di halaman</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>NVDA: tekan NVDA+Insert+F7, pilih bagian Landmarks, hitung jumper banner</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2702,9 +2755,9 @@
           <t>Ada tepat satu judul utama (h1)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>DevTools: ketik document.querySelectorAll('h1').length di Console, atau NVDA tekan H</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -2713,6 +2766,11 @@
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2727,9 +2785,9 @@
           <t>Urutan judul tidak melompat-lompat</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>NVDA: tekan H berulang, tulis urutan judul yang terdengar</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -2738,6 +2796,11 @@
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2752,9 +2815,9 @@
           <t>Semua tautan punya tulisan yang menjelaskan tujuan</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>NVDA: tekan K, baca semua nama tautan tanpa melihat layar</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -2763,6 +2826,11 @@
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2777,17 +2845,22 @@
           <t>Logo utama terbaca oleh screen reader</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>NVDA: tekan K, dengarkan tautan pertama</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2802,9 +2875,9 @@
           <t>Semua tombol dan isian punya nama yang terbaca</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>DevTools tab Accessibility: klik Inspect, baca Computed Properties (Name, Role)</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -2812,7 +2885,12 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -2827,17 +2905,22 @@
           <t>Semua isian formulir punya label yang terhubung</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>DevTools: klik kanan isian, pilih Inspect, cari &lt;label for=...&gt;</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -2852,17 +2935,22 @@
           <t>Pesan kesalahan formulir dibacakan screen reader</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>NVDA + Speech Viewer (NVDA+F5) untuk merekam apa yang diucapkan</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
@@ -2877,9 +2965,9 @@
           <t>Warna teks utama cukup kontras dengan latar</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>DevTools: klik kanan teks, Inspect &gt; eyedropper. Catat 2 kode warna.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -2888,6 +2976,11 @@
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2902,9 +2995,9 @@
           <t>Teks masih terbaca saat halaman dizoom 200 persen</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Browser: tekan Ctrl lalu + dua kali</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -2913,6 +3006,11 @@
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2927,17 +3025,22 @@
           <t>Tidak ada gulir ke samping saat layar 320 piksel</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>DevTools: tekan Ctrl+Shift+M, set lebar 320 piksel</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2952,9 +3055,9 @@
           <t>Gambar punya keterangan yang benar</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>DevTools Inspect + NVDA tekan G untuk pindah ke gambar</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -2963,6 +3066,11 @@
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2977,17 +3085,22 @@
           <t>Video punya subtitle Bahasa Indonesia yang cocok dengan suara</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Pemutar YouTube: klik tombol CC, putar di detik 0, tengah, dan hampir akhir</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
@@ -3002,17 +3115,22 @@
           <t>File PDF punya judul dan bahasa yang terisi</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Adobe Acrobat Reader: Tools &gt; Accessibility &gt; Check PDF Accessibility</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
@@ -3027,9 +3145,9 @@
           <t>Tidak ada dua gambar atau cahaya yang berkedip cepat</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Pemutar video + Windows: Settings &gt; Accessibility &gt; Visual effects &gt; Animation effects OFF</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -3038,6 +3156,11 @@
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -3052,17 +3175,22 @@
           <t>Bahasa halaman ditandai dengan benar (id-ID)</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>DevTools: klik kanan html, Inspect, lihat atribut lang</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -3077,17 +3205,22 @@
           <t>Ada cara melapor masalah aksesibilitas</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Cek kaki halaman. NVDA untuk memastikan tautannya terbaca.</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -3098,10 +3231,6 @@
         <is>
           <t>Jumlah gagal</t>
         </is>
-      </c>
-      <c r="C27">
-        <f>COUNTIF(C4:C25,"G")</f>
-        <v/>
       </c>
       <c r="D27">
         <f>COUNTIF(D4:D25,"G")</f>
@@ -3111,16 +3240,16 @@
         <f>COUNTIF(E4:E25,"G")</f>
         <v/>
       </c>
+      <c r="F27">
+        <f>COUNTIF(F4:F25,"G")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Jumlah sudah diuji</t>
         </is>
-      </c>
-      <c r="C28">
-        <f>COUNTIF(C4:C25,"L")+COUNTIF(C4:C25,"G")</f>
-        <v/>
       </c>
       <c r="D28">
         <f>COUNTIF(D4:D25,"L")+COUNTIF(D4:D25,"G")</f>
@@ -3130,10 +3259,14 @@
         <f>COUNTIF(E4:E25,"L")+COUNTIF(E4:E25,"G")</f>
         <v/>
       </c>
+      <c r="F28">
+        <f>COUNTIF(F4:F25,"L")+COUNTIF(F4:F25,"G")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>